<commit_message>
LLM-readiness + vendor-risk depth: homepage agent hub, changelog, JSON-LD, procurement templates
- Homepage: add 'For LLMs & agents' resource hub (llms.txt, full-text, data
  index, knowledge graph, schema viewer, retrieval validation).
- Add /changelog/ with release-grouped entries; link from footer.
- Add schema.org JSON-LD to both vendor-risk pages (TechArticle, HowTo).
- Vendor-risk export templates: copy-ready contract clauses and RFP questions
  on-page, plus Attestation Mapping, Contract Clauses, and RFP Questions tabs
  in the workpaper xlsx.
- Update llms.txt, llms-full.txt, sitemap.xml for the changelog.
</commit_message>
<xml_diff>
--- a/tools/vendor-risk/how-to/vendor-risk-workpaper.xlsx
+++ b/tools/vendor-risk/how-to/vendor-risk-workpaper.xlsx
@@ -12,6 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accountability Split" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attestation Reference" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Bank" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attestation Mapping" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract Clauses" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFP Questions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Question Bank'!$A$1:$K$38</definedName>
@@ -102,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +143,11 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2964,4 +2972,407 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Attestation</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Evidence it can satisfy</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>AI-specific gaps to ask separately</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>SOC 2 Type II</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Tenant isolation, encryption, access control, incident response, availability, and confidentiality controls operating over a period.</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Model behavior, bias, prompt injection, autonomy, training-data provenance, IP indemnity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>ISO/IEC 27001</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>An information security management system covering most platform and data-handling questions.</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>AI governance, model lifecycle, agent authorization, retrieval integrity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>ISO/IEC 42001</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>AI governance, AI risk management, model lifecycle, and responsible-AI controls. The AI-specific signal.</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Point-in-time security control testing; does not replace SOC 2 or ISO 27001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>ISO 9001</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Quality management for labeling and annotation accuracy.</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Security, data protection, and AI-specific risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>FedRAMP</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Cloud platform security at a defined US federal impact level.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>AI governance and model behavior beyond the platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>NIST AI RMF</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>A structured AI risk-management process, mapped to govern, map, measure, manage.</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Independent certification; verify it is audited, not just self-asserted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>EU AI Act</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Risk categorization and the legal obligations for in-scope systems.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Security and quality control evidence.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="104" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Clause</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Draft text (edit bracketed terms; have counsel review)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Shared-responsibility matrix</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Vendor shall maintain and attach as an exhibit a responsibility matrix that assigns one accountable party to each control across the applicable SRF layers (L1 to L5). Where a control is jointly operated, the matrix shall separate the portion Vendor controls from the portion [Customer] controls and assign each to a single owner. Vendor shall not characterize any control as 'shared' without this split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Data use and no training on customer data</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Vendor shall not use [Customer] data, prompts, inputs, or outputs to train, fine-tune, or evaluate any model that is made available to other customers, and shall not retain such data beyond the period required to deliver the service. Vendor shall provide written confirmation of this control and evidence of technical enforcement on request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Sub-processors, residency, and change notice</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Vendor shall maintain a current list of all sub-processors, including any model, infrastructure, and labeling providers, with each provider's geographic location and data role. Vendor shall process [Customer] data only in [permitted regions] and shall give [Customer] at least [30] days' written notice before adding or replacing a sub-processor, changing a processing location, or changing the model that powers the service, with a right to object.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>AI liability and IP indemnification</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Vendor shall indemnify [Customer] against third-party claims that the service's AI output infringes intellectual property rights. The parties shall allocate liability for losses arising from AI-generated output, including erroneous, harmful, or non-compliant output, as set out in [Schedule X], and such liability shall not be excluded by general limitations on consequential damages to the extent it arises from Vendor's failure to meet the controls in this agreement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Agentic controls and kill-switch</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>For any autonomous or agentic capability, Vendor shall provide [Customer] with configurable controls over autonomy level and human override, scope and rate limits on tool and action use, the ability to require human approval for [defined high-impact actions], a complete audit trail of agent actions, and a documented mechanism to immediately suspend agent activity. Vendor shall not change default autonomy or override settings without prior written notice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Continuous evidence, re-assessment, and secure deletion</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Vendor shall provide evidence that the controls in this agreement are operating, on a [continuous / quarterly] basis rather than only at point-in-time, and shall permit [Customer] to re-assess on any material change to the model, sub-processors, or autonomy configuration. On termination, Vendor shall securely delete all [Customer] data and provide a certificate of deletion within [30] days.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="104" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>AI-specific RFP question</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Vendor response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Which SRF layers does your offering touch (L1 to L5), and what is your operating model (AI-SaaS, AI-PaaS, Agent-PaaS, IaaS)?</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr"/>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Provide a responsibility matrix stating which controls you own and which remain with us.</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>List the foundation models and sub-processors behind the service, with their geographic locations and data roles.</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr"/>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Confirm in writing that our data, prompts, and outputs are not used to train shared models, and describe how this is enforced.</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Provide your current attestations (SOC 2 Type II, ISO/IEC 27001, ISO/IEC 42001) and, for AI governance, your ISO 42001 certification or NIST AI RMF profile.</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Describe your defenses against prompt injection, including indirect injection from retrieved content or tool output.</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr"/>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Provide model and weight provenance, signing, and an AI bill of materials (AIBOM).</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr"/>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>For agentic features, state the autonomy levels and human-override tiers supported, the permission model, and the kill-switch mechanism.</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr"/>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Describe how you notify customers of model, sub-processor, and autonomy changes, and the notice period.</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr"/>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Provide your data-retention and secure-deletion policy, including certificates of destruction on exit.</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>